<commit_message>
Substituted LTE module 13 with module 5
Substituted LTE module 13 with module 5, changed the information on the inventory form.
</commit_message>
<xml_diff>
--- a/Sensor Box Deployment Inventory /SensorBox_Component_Tracker.xlsx
+++ b/Sensor Box Deployment Inventory /SensorBox_Component_Tracker.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kriishhate/GitHub/CommonSENSES/Sensor Box Deployment Inventory /"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/allensong/Documents/GitHub/CommonSENSES/Sensor Box Deployment Inventory /"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C00D8A8-51E6-9A49-A93F-7B738A546C32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62C8F422-65E6-C44D-98E1-E36B19132724}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6920" yWindow="1840" windowWidth="27640" windowHeight="16940" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
   </bookViews>
@@ -92,9 +92,6 @@
     <t>e00fce68cb9b730d1fdeb3ac</t>
   </si>
   <si>
-    <t>e00fce682af8b21e177ae3ac</t>
-  </si>
-  <si>
     <t>e00fce682c905f7d061a9fc5</t>
   </si>
   <si>
@@ -384,6 +381,9 @@
   </si>
   <si>
     <t>55</t>
+  </si>
+  <si>
+    <t>e00fce6859cf08424ab70193</t>
   </si>
 </sst>
 </file>
@@ -800,13 +800,13 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B2" t="s">
         <v>6</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D2" t="s">
         <v>4</v>
@@ -817,13 +817,13 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B3" t="s">
         <v>7</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D3" t="s">
         <v>4</v>
@@ -834,13 +834,13 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B4" t="s">
         <v>8</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D4" t="s">
         <v>4</v>
@@ -851,13 +851,13 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D5" t="s">
         <v>4</v>
@@ -868,13 +868,13 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B6" t="s">
         <v>10</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D6" t="s">
         <v>4</v>
@@ -885,13 +885,13 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B7" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D7" t="s">
         <v>4</v>
@@ -902,13 +902,13 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B8" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D8" t="s">
         <v>4</v>
@@ -919,13 +919,13 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B9" t="s">
         <v>13</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D9" t="s">
         <v>4</v>
@@ -936,13 +936,13 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B10" t="s">
         <v>14</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D10" t="s">
         <v>4</v>
@@ -953,13 +953,13 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B11" t="s">
         <v>15</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D11" t="s">
         <v>4</v>
@@ -970,13 +970,13 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B12" t="s">
         <v>16</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D12" t="s">
         <v>4</v>
@@ -987,13 +987,13 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B13" t="s">
         <v>17</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D13" t="s">
         <v>4</v>
@@ -1004,30 +1004,30 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B14" t="s">
-        <v>18</v>
+        <v>115</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D14" t="s">
         <v>4</v>
       </c>
       <c r="E14" s="2">
-        <v>45793</v>
+        <v>45826</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B15" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D15" t="s">
         <v>4</v>
@@ -1038,13 +1038,13 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B16" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D16" t="s">
         <v>4</v>
@@ -1055,13 +1055,13 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B17" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D17" t="s">
         <v>4</v>
@@ -1072,13 +1072,13 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B18" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D18" t="s">
         <v>4</v>
@@ -1089,13 +1089,13 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B19" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D19" t="s">
         <v>4</v>
@@ -1106,13 +1106,13 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B20" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D20" t="s">
         <v>4</v>
@@ -1123,13 +1123,13 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B21" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D21" t="s">
         <v>4</v>
@@ -1140,13 +1140,13 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D22" t="s">
         <v>4</v>
@@ -1157,13 +1157,13 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B23" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D23" t="s">
         <v>4</v>
@@ -1174,13 +1174,13 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B24" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D24" t="s">
         <v>4</v>
@@ -1191,13 +1191,13 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B25" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D25" t="s">
         <v>4</v>
@@ -1208,13 +1208,13 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B26" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D26" t="s">
         <v>4</v>
@@ -1225,13 +1225,13 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D27" t="s">
         <v>4</v>
@@ -1242,13 +1242,13 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B28" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D28" t="s">
         <v>4</v>
@@ -1259,13 +1259,13 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B29" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D29" t="s">
         <v>4</v>
@@ -1276,13 +1276,13 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B30" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D30" t="s">
         <v>4</v>
@@ -1293,13 +1293,13 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B31" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D31" t="s">
         <v>4</v>
@@ -1310,13 +1310,13 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B32" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D32" t="s">
         <v>4</v>
@@ -1327,13 +1327,13 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B33" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D33" t="s">
         <v>4</v>
@@ -1344,13 +1344,13 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B34" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D34" t="s">
         <v>4</v>
@@ -1361,13 +1361,13 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B35" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D35" t="s">
         <v>4</v>
@@ -1378,13 +1378,13 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B36" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D36" t="s">
         <v>4</v>
@@ -1395,13 +1395,13 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B37" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D37" t="s">
         <v>4</v>
@@ -1412,13 +1412,13 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B38" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D38" t="s">
         <v>4</v>
@@ -1429,13 +1429,13 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B39" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D39" t="s">
         <v>4</v>
@@ -1446,13 +1446,13 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B40" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D40" t="s">
         <v>4</v>
@@ -1463,13 +1463,13 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B41" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D41" t="s">
         <v>4</v>
@@ -1480,13 +1480,13 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B42" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D42" t="s">
         <v>4</v>
@@ -1497,13 +1497,13 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B43" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D43" t="s">
         <v>4</v>
@@ -1514,13 +1514,13 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B44" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D44" t="s">
         <v>4</v>
@@ -1531,13 +1531,13 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B45" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D45" t="s">
         <v>4</v>
@@ -1548,13 +1548,13 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B46" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D46" t="s">
         <v>4</v>
@@ -1565,13 +1565,13 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B47" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D47" t="s">
         <v>4</v>
@@ -1582,13 +1582,13 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B48" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D48" t="s">
         <v>4</v>
@@ -1599,13 +1599,13 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B49" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D49" t="s">
         <v>4</v>
@@ -1616,13 +1616,13 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B50" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D50" t="s">
         <v>4</v>
@@ -1633,13 +1633,13 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A51" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B51" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D51" t="s">
         <v>4</v>
@@ -1650,13 +1650,13 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B52" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D52" t="s">
         <v>4</v>
@@ -1667,13 +1667,13 @@
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A53" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B53" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D53" t="s">
         <v>4</v>
@@ -1684,13 +1684,13 @@
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A54" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B54" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D54" t="s">
         <v>4</v>
@@ -1701,13 +1701,13 @@
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A55" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B55" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D55" t="s">
         <v>4</v>
@@ -1718,13 +1718,13 @@
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A56" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B56" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D56" t="s">
         <v>4</v>

</xml_diff>